<commit_message>
add recommendation summary field data check from the database
</commit_message>
<xml_diff>
--- a/docs/report3/IACAssessmentTemplate.v2.1.xlsx
+++ b/docs/report3/IACAssessmentTemplate.v2.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lsumail2-my.sharepoint.com/personal/chaowang_lsu_edu/Documents/LSU-IAC/00-FY 2024/Manufacturing Facility/LS2503 - LaShip/Draft Report/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/achowd6/Codes/itac-report-validator/docs/report3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="470" documentId="14_{1867FAE8-2998-472C-95D2-9783179EDA43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6BCB4C3-90B3-C640-8243-6754B74B520D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F7A9305-4FE2-1A47-B1EF-22550817F922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14780" yWindow="920" windowWidth="14460" windowHeight="18040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1073,10 +1073,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -2520,7 +2516,7 @@
         <v>None</v>
       </c>
       <c r="W4" s="30">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="X4" s="30">
         <v>40</v>
@@ -5985,7 +5981,7 @@
       </c>
       <c r="W45">
         <f>'Recommendation Info'!W4</f>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="X45">
         <f>'Recommendation Info'!X4</f>

</xml_diff>